<commit_message>
Textura en reporte de clientes v1
</commit_message>
<xml_diff>
--- a/tests/text archivo ej 01.xlsx
+++ b/tests/text archivo ej 01.xlsx
@@ -236,7 +236,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -268,6 +268,13 @@
     <font>
       <b val="true"/>
       <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -315,7 +322,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -334,6 +341,14 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -356,37 +371,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18A303"/>
+        <a:srgbClr val="18a303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369A3"/>
+        <a:srgbClr val="0369a3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A33E03"/>
+        <a:srgbClr val="a33e03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8E03A3"/>
+        <a:srgbClr val="8e03a3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="C99C00"/>
+        <a:srgbClr val="c99c00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="C9211E"/>
+        <a:srgbClr val="c9211e"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000EE"/>
+        <a:srgbClr val="0000ee"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551A8B"/>
+        <a:srgbClr val="551a8b"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -459,7 +474,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O40"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19.2"/>
@@ -572,11 +587,11 @@
       <c r="M3" s="1" t="n">
         <v>61</v>
       </c>
-      <c r="N3" s="1" t="n">
-        <v>358</v>
-      </c>
-      <c r="O3" s="1" t="n">
-        <v>1442</v>
+      <c r="N3" s="5" t="n">
+        <v>21480</v>
+      </c>
+      <c r="O3" s="5" t="n">
+        <v>86520</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -619,11 +634,11 @@
       <c r="M4" s="1" t="n">
         <v>59</v>
       </c>
-      <c r="N4" s="1" t="n">
-        <v>362</v>
-      </c>
-      <c r="O4" s="1" t="n">
-        <v>1438</v>
+      <c r="N4" s="5" t="n">
+        <v>21720</v>
+      </c>
+      <c r="O4" s="5" t="n">
+        <v>86280</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -666,11 +681,11 @@
       <c r="M5" s="1" t="n">
         <v>60</v>
       </c>
-      <c r="N5" s="1" t="n">
-        <v>359</v>
-      </c>
-      <c r="O5" s="1" t="n">
-        <v>1441</v>
+      <c r="N5" s="5" t="n">
+        <v>21540</v>
+      </c>
+      <c r="O5" s="5" t="n">
+        <v>86460</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -713,11 +728,11 @@
       <c r="M6" s="1" t="n">
         <v>61</v>
       </c>
-      <c r="N6" s="1" t="n">
-        <v>358</v>
-      </c>
-      <c r="O6" s="1" t="n">
-        <v>1438</v>
+      <c r="N6" s="5" t="n">
+        <v>21480</v>
+      </c>
+      <c r="O6" s="5" t="n">
+        <v>86280</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -760,11 +775,11 @@
       <c r="M7" s="1" t="n">
         <v>62</v>
       </c>
-      <c r="N7" s="1" t="n">
-        <v>361</v>
-      </c>
-      <c r="O7" s="1" t="n">
-        <v>1439</v>
+      <c r="N7" s="5" t="n">
+        <v>21660</v>
+      </c>
+      <c r="O7" s="5" t="n">
+        <v>86340</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -807,11 +822,11 @@
       <c r="M8" s="1" t="n">
         <v>58</v>
       </c>
-      <c r="N8" s="1" t="n">
-        <v>357</v>
-      </c>
-      <c r="O8" s="1" t="n">
-        <v>1443</v>
+      <c r="N8" s="5" t="n">
+        <v>21420</v>
+      </c>
+      <c r="O8" s="5" t="n">
+        <v>86580</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -854,11 +869,11 @@
       <c r="M9" s="1" t="n">
         <v>60</v>
       </c>
-      <c r="N9" s="1" t="n">
-        <v>363</v>
-      </c>
-      <c r="O9" s="1" t="n">
-        <v>1440</v>
+      <c r="N9" s="5" t="n">
+        <v>21780</v>
+      </c>
+      <c r="O9" s="5" t="n">
+        <v>86400</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -901,11 +916,11 @@
       <c r="M10" s="1" t="n">
         <v>61</v>
       </c>
-      <c r="N10" s="1" t="n">
-        <v>360</v>
-      </c>
-      <c r="O10" s="1" t="n">
-        <v>1437</v>
+      <c r="N10" s="5" t="n">
+        <v>21600</v>
+      </c>
+      <c r="O10" s="5" t="n">
+        <v>86220</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -948,11 +963,11 @@
       <c r="M11" s="1" t="n">
         <v>59</v>
       </c>
-      <c r="N11" s="1" t="n">
-        <v>358</v>
-      </c>
-      <c r="O11" s="1" t="n">
-        <v>1442</v>
+      <c r="N11" s="5" t="n">
+        <v>21480</v>
+      </c>
+      <c r="O11" s="5" t="n">
+        <v>86520</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -995,11 +1010,11 @@
       <c r="M12" s="1" t="n">
         <v>60</v>
       </c>
-      <c r="N12" s="1" t="n">
-        <v>361</v>
-      </c>
-      <c r="O12" s="1" t="n">
-        <v>1444</v>
+      <c r="N12" s="5" t="n">
+        <v>21660</v>
+      </c>
+      <c r="O12" s="5" t="n">
+        <v>86640</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1042,11 +1057,11 @@
       <c r="M13" s="1" t="n">
         <v>61</v>
       </c>
-      <c r="N13" s="1" t="n">
-        <v>359</v>
-      </c>
-      <c r="O13" s="1" t="n">
-        <v>1439</v>
+      <c r="N13" s="5" t="n">
+        <v>21540</v>
+      </c>
+      <c r="O13" s="5" t="n">
+        <v>86340</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1089,12 +1104,90 @@
       <c r="M14" s="1" t="n">
         <v>60</v>
       </c>
-      <c r="N14" s="1" t="n">
-        <v>360</v>
-      </c>
-      <c r="O14" s="1" t="n">
-        <v>1441</v>
-      </c>
+      <c r="N14" s="5" t="n">
+        <v>21600</v>
+      </c>
+      <c r="O14" s="5" t="n">
+        <v>86460</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K28" s="6"/>
+      <c r="L28" s="6"/>
+      <c r="M28" s="6"/>
+      <c r="N28" s="6"/>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K29" s="5"/>
+      <c r="L29" s="5"/>
+      <c r="M29" s="5"/>
+      <c r="N29" s="5"/>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K30" s="5"/>
+      <c r="L30" s="5"/>
+      <c r="M30" s="5"/>
+      <c r="N30" s="5"/>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K31" s="5"/>
+      <c r="L31" s="5"/>
+      <c r="M31" s="5"/>
+      <c r="N31" s="5"/>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K32" s="5"/>
+      <c r="L32" s="5"/>
+      <c r="M32" s="5"/>
+      <c r="N32" s="5"/>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K33" s="5"/>
+      <c r="L33" s="5"/>
+      <c r="M33" s="5"/>
+      <c r="N33" s="5"/>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K34" s="5"/>
+      <c r="L34" s="5"/>
+      <c r="M34" s="5"/>
+      <c r="N34" s="5"/>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K35" s="5"/>
+      <c r="L35" s="5"/>
+      <c r="M35" s="5"/>
+      <c r="N35" s="5"/>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K36" s="5"/>
+      <c r="L36" s="5"/>
+      <c r="M36" s="5"/>
+      <c r="N36" s="5"/>
+    </row>
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K37" s="5"/>
+      <c r="L37" s="5"/>
+      <c r="M37" s="5"/>
+      <c r="N37" s="5"/>
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K38" s="5"/>
+      <c r="L38" s="5"/>
+      <c r="M38" s="5"/>
+      <c r="N38" s="5"/>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K39" s="5"/>
+      <c r="L39" s="5"/>
+      <c r="M39" s="5"/>
+      <c r="N39" s="5"/>
+    </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K40" s="5"/>
+      <c r="L40" s="5"/>
+      <c r="M40" s="5"/>
+      <c r="N40" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>